<commit_message>
Merge the three correspondence tables into a single sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qax4kDvA5VYNQopw9xUKNT
</commit_message>
<xml_diff>
--- a/جداول_الملف.xlsx
+++ b/جداول_الملف.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="جدول 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="جدول 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="جدول 3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المراسلات" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'المراسلات'!$A$1:$F$38</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,18 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -42,7 +37,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -54,8 +49,13 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -77,19 +77,65 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -457,831 +503,921 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>بيان المراسلات الصادرة من المدعية بشأن الأعمال القانونية المتعلقة بالصفقة محل التداعي</t>
-        </is>
-      </c>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الراسل وصفته</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المرسل إليه وصفته</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>مضمون الرسالة</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>المستند المؤيد / ملاحظة</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الجدول 1: بيان المراسلات الصادرة من المدعية بشأن الأعمال القانونية المتعلقة بالصفقة محل التداعي</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>التاريخ</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>الراسل وصفته</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>المرسل اليه وصفتة</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>مضمون الرسالة</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>المستند المؤيد لذلك</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>20/12/2025</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>إرسال نسخة منقحة من اتفاقية الأتعاب عقب مراجعة تعليقات المدعى عليها على مسودتها</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>صورة البريد الإلكتروني المؤرخ 20/12/2025</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>20/12/2025</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>إرسال نسخة منقحة من اتفاقية الأتعاب عقب مراجعة تعليقات المدعى عليها على مسودتها</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>صورة البريد الإلكتروني المؤرخ 20/12/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>22/12/2025
 الساعة 9:29 صباحاً</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>إضافة أحكام ضريبة القيمة المضافة، وإعداد النسخة العربية من اتفاقية الأتعاب، وإرسالها للتوقيع</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 22/12/2025،الساعة 9:29 صباحاً</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>22/12/2025
 الساعة 4:55 مساءً</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>طلب إعادة مسح الاتفاقية الموقعة بما يكفل وضوح صفحاتها وظهور النص كاملاً</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 22/12/2025،الساعة 4:55 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>22/12/2025
 الساعة 6:18 مساءً</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>إرسال اتفاقية الأتعاب الموقعة من جانب المدعية</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 22/12/2025،الساعة 6:18 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>23/12/2025
 الساعة 1:29 مساءً</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>إبداء الرأي القانوني بشأن ورقة الشروط، ورصد اختلاف نسب الحصص عن الشروط السابقة، والتوجيه إلى التفاوض بشأنها</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني الساعة 1:29 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>26/12/2025
 الساعة 3:42 مساءً</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>الإفادة بمتابعة الفريق القانوني للبائع والاستمرار في إعداد مسودة اتفاقية عدم الإفصاح</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 26/12/2025،الساعة 3:42 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>29/12/2025
 الساعة 1:08 مساءً</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>تسليم مسودة اتفاقية عدم إفصاح ثنائية اللغة لتنظيم تبادل المعلومات وسريتها دون إلزام بإتمام الصفقة</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 29/12/2025،الساعة 1:08 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>05/01/2026
 الساعة 12:00 ظهراً</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>تأكيد استلام ورقة الشروط ومرفقاتها؛ وهي مراسلة متابعة واستلام وليست بذاتها تسليماً لرأي قانوني</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 05/01/2026 الساعة 12:00 ظهراً</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>12/01/2026
 الساعة 8:56 مساءً</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>التنبيه إلى نقص مستندات الأرض، واقتراح صياغة مذكرة تفاهم عامة أو مشروطة لحين الإفصاح الكامل عن المستندات</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 12/01/2026 الساعة 8:56 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>15/01/2026
 الساعة 5:30 مساءً</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>عرض ملاحظات قانونية تفصيلية ومسودة بديلة تتناول الإلزام والسرية والضمانات والدفع والحوكمة وتسوية المنازعات</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 15/01/2026،الساعة 5:30 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>15/01/2026
 الساعة 5:32 مساءً</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>تسليم مسودة مذكرة التفاهم التي أعدتها المدعية</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 15/01/2026 الساعة 5:32 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>16/01/2026
 الساعة 1:58 مساءً</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>تأكيد مراجعة تعليقات المدعى عليها والشروع في إعادة صياغة المسودة وفق تلك التعليقات</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 16/01/2026 الساعة 1:58 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>19/01/2026
 الساعة 7:33 مساءً</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>إرسال النسخة الرابعة المعدلة من مذكرة التفاهم بصيغتي Word وPDF، وطلب إحالة النسخة الأحدث إلى البائع</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 19/01/2026 الساعة 7:33 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>20/01/2026
 الساعة 7:42 مساءً</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>إرسال النسخة الخامسة من مذكرة التفاهم بصيغتيها النظيفة والمتعقبة، مع الإشارة إلى بيانات البائع المطلوب استكمالها</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 20/01/2026 الساعة 7:42 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>21/01/2026
 الساعة 11:57 صباحاً</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>إعادة إرسال مذكرة التفاهم عقب طلب مراجعتها، تمهيداً لاجتماع اليوم ذاته</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 21/01/2026 الساعة 11:57 صباحاً</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>26/01/2026
 الساعة 8:48 مساءً</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>بيان خطوات إحالة مسودة اتفاقية التطوير، وطلب المستندات ومتابعة إجراءات الامتثال والتحقق من نموذج البيع والشراء</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 26/01/2026،الساعة 8:48 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>26/02/2026
 الساعة 12:19 ظهراً</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>تأكيد طلب مستندات الصفة والسلطة والملكية والاستحقاق من الشركة القابضة، وبيان ضرورة فحصها قبل التوقيع</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني الساعة 12:19 ظهراً</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>09/03/2026
 الساعة 12:40 ظهراً</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>تسليم رأي قانوني مكتوب ومفصل بشأن اتفاقية شراء الأرض، متضمناً الإجابة عن الأسئلة القانونية المطروحة</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 09/03/2026 الساعة 12:40 ظهراً</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>11/03/2026
 الساعة 9:30 مساءً</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>إرسال المراجع التشريعية والتنظيمية الرسمية المتعلقة بالتملك والتسجيل استكمالاً للرأي القانوني المطلوب</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 11/03/2026 الساعة 9:30 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>11/03/2026
 الساعة 9:46 مساءً</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>إرسال ملحق اتفاقية الأتعاب بصيغتي Word وPDF للمراجعة والتوقيع</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 11/03/2026 الساعة 9:46 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>12/03/2026
 الساعة 2:27 مساءً</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>تقديم تأكيد قانوني بشأن أهلية المشتري للتملك، مع بيان المراجع التي استند إليها الرأي</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 12/03/2026،الساعة 2:27 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>16/04/2026
 الساعة 6:19 مساءً</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع والمدعى عليها</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>التدخل في تنسيق موعد الاجتماع بشأن الصفقة، واقتراح إعادة جدولته لعدم توافر السيد فيكتور البتيف</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 16/04/2026،الساعة 6:19 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>17/04/2026
 الساعة 9:31 مساءً</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع والمدعى عليها</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>مواصلة تنسيق موعد الاجتماع وتأكيد استمرار الاهتمام بالأرض محل الصفقة</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 17/04/2026 الساعة 9:31 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>24/04/2026
 الساعة 7:24 مساءً</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>إبداء الرأي القانوني بشأن مخاطر التمديد الضمني والعرض الملزم والإقرار بالمراسلات، واقتراح صياغة تحافظ على المرونة التفاوضية</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 24/04/2026 الساعة 7:24 مساءً</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>30/04/2026
 الساعة 6:41 مساءً</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>المدعى عليها</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>المدعى عليها</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>تسليم نتيجة المراجعة القانونية والرأي النهائي بشأن الملحق المتعلق بالصفقة، والتوصية بتوضيح الجاهزية لنقل الملكية</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ 30/04/2026 الساعة 6:41 مساءً</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>وكذلك نرفق للخبرة الموقرة ، جدول اعمال المدعية خلال يوم 30/4/2026 
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>جدول 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>الجدول 2: وكذلك نرفق للخبرة الموقرة ، جدول اعمال المدعية خلال يوم 30/4/2026 
 وجدول اعمال ما بعد 30/4/2026 حتي 19/5/2026</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>التاريخ</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>الراسل</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>المرسل اليه</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>مضمون الرسالة</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>المستند المؤيد</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>30/4/2026
 الساعة10:30 صباحاً</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>المدعي عليها</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>ايميل من المدعي عليها الي المدعية مرفق به مسودة الاتفاقية التكميلية الخاصة بشراء الأرض إلى المدعية لمراجعتها قانونيًا وإبداء ملاحظاتها عليها، مع طلب سرعة الرد قبل نهاية اليوم نظرًا لضيق الوقت</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المؤرخ
 30/4/2026
@@ -1290,307 +1426,309 @@
 والمرفق بمستندات الدعوي ومذكرة اليوم</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>جدول 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>30/4/2026
 الساعة14:40 مساءاً</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>المدعي عليها</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>صورة البريد الإلكتروني المتضمن طلب مراجعة الاتفاقية قانونيًا في هيكل المعاملة، والمرفق به مستند يفيد تغيير اسم المشتري إلى شركة أرسنال إيست للتطوير العقاري المحدودة بصفتها المشتري الجديد، بما يثبت استمرار الاستعانة بالمدعية لمراجعة المستندات القانونية ومتابعة التعديلات المتعلقة بأطراف صفقة شراء الأرض النهائية</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>البريد الالكتروني الرقيم 61- المؤرخ 30/4/2026 الساعة 14:40
 والمرفق بمستندات الدعوي ومذكرة اليوم</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>جدول 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>30/4/2026
 الساعة 5:23 مساءاً</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>المدعية</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>المدعية</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>المدعي عليها</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>رداً من المدعية علي ايميل المدعي عليهم رقم (61) وتم عمل المطلوب من حيث فحص ومراجعة قانونية لأتفاقية البيع النهائي وعلم المدعية بأسم المشتري الجديد</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>البريد الالكتروني رقم(62)-المؤرخ30/4/2026
  رداً من المدعية علي طلب المراجعة من المدعي عليهم
 والمرفق بمستندات الدعوي ومذكرة اليوم</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26.5" customWidth="1" min="2" max="2"/>
-    <col width="26.5" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>الثابت من المراسلات الإلكترونية والمستندات المقدمة أن دور المدعية لم ينقطع عند تاريخ 30/04/2026، وإنما استمرت صلتها المهنية بصفقة شراء الأرض، حيث حرص المدعى عليهم والأطراف المعنية بالصفقة على إدراج المدعية ضمن المراسلات الإلكترونية المتبادلة خلال الفترة من 03/05/2026 حتى 19/05/2026، وإحاطتها بالتطورات الجوهرية المتعلقة باستكمال الصفقة، بما في ذلك توقيع ملحق الاتفاقية، وتغيير المشتري، ومتابعة الإجراءات القانونية والتنظيمية مع المطور الرئيسي، واستصدار شهادة عدم الممانعة، وتداول الاتفاقيات والمستندات اللازمة لاستكمال إجراءات نقل الملكية،  ولا يمكن النظر إلى استمرار إدراج المدعية ضمن تلك المراسلات بمعزل عن الأعمال القانونية التي سبق أن باشرتها بشأن ذات الصفقة، إذ لم تكن المدعية طرفًا أجنبيًا عن الاتفاقية أو مجرد جهة أُدرجت مصادفة ضمن المراسلات، وإنما كانت المدعية هي التي تولت مراجعة الاتفاقيات وإبداء الملاحظات القانونية بشأنها بما فيها واهمها ( الاتفاقية النهائية التي راجعتها المدعية بتاريخ 30/4/2026) ، الأمر الذي يثبت ويؤكد استمرار إحاطتها بالاجراءات المتعلقة بتطورات الصفقة، ويؤكد اتصال الأعمال القانونية التي قدمتها بالإجراءات اللاحقة التي اتخذها أطراف الصفقة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>التاريخ</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>الراسل</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>المرسل اليه</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>بيان الموضوع</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>المدعية (سي سي )</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>جدول 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>الجدول 3: الثابت من المراسلات الإلكترونية والمستندات المقدمة أن دور المدعية لم ينقطع عند تاريخ 30/04/2026، وإنما استمرت صلتها المهنية بصفقة شراء الأرض، حيث حرص المدعى عليهم والأطراف المعنية بالصفقة على إدراج المدعية ضمن المراسلات الإلكترونية المتبادلة خلال الفترة من 03/05/2026 حتى 19/05/2026، وإحاطتها بالتطورات الجوهرية المتعلقة باستكمال الصفقة، بما في ذلك توقيع ملحق الاتفاقية، وتغيير المشتري، ومتابعة الإجراءات القانونية والتنظيمية مع المطور الرئيسي، واستصدار شهادة عدم الممانعة، وتداول الاتفاقيات والمستندات اللازمة لاستكمال إجراءات نقل الملكية،  ولا يمكن النظر إلى استمرار إدراج المدعية ضمن تلك المراسلات بمعزل عن الأعمال القانونية التي سبق أن باشرتها بشأن ذات الصفقة، إذ لم تكن المدعية طرفًا أجنبيًا عن الاتفاقية أو مجرد جهة أُدرجت مصادفة ضمن المراسلات، وإنما كانت المدعية هي التي تولت مراجعة الاتفاقيات وإبداء الملاحظات القانونية بشأنها بما فيها واهمها ( الاتفاقية النهائية التي راجعتها المدعية بتاريخ 30/4/2026) ، الأمر الذي يثبت ويؤكد استمرار إحاطتها بالاجراءات المتعلقة بتطورات الصفقة، ويؤكد اتصال الأعمال القانونية التي قدمتها بالإجراءات اللاحقة التي اتخذها أطراف الصفقة.</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>03/05/2026</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>ممثل المدعي عليها 
 والمدعي عليه الثالث 
 فيكتور لابتيف</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع
 خالد أحمد الهاشمي</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>مراسلة صادرة من ممثل المدعى عليها الأولى إلى ممثل البائع، مرفقًا بها الملحق التكميلي المؤرخ 3/5/2026 لاتفاقية شراء الارض المؤرخة 9/3/2026 موقعًا من جانب المشتري (المدعى عليها الأولى)، مع طلب توقيعه وإعادة النسخة الموقعة خلال 48 ساعة والإشارة إلى إمكانية بحث شراكة مستقبلية بنسبتي 60% و 40%</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>والمدعية (سي سي ) بهذا الايميل</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>جدول 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>05/05/2026</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع السيد 
 ( خالد أحمد الهاشمي )</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>ممثل المدعي عليها 
 والمدعي عليه الثالث 
 فيكتور لابتيف</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>إرسال نسخة الاتفاقية النهائية  الموقعة، وتأكيد تقديم طلب شهادة عدم الممانعة إلى مبادلة، وبيان متطلبات اعرف عميلك المستندات اللازمة لاستكمال إجراءات نقل الملكية</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>والمدعية (سي سي ) بهذا الايميل</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>جدول 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>08/05/2026</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع السيد 
 ( خالد أحمد الهاشمي )</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>ممثل المدعي عليها 
 والمدعي عليه الثالث 
 فيكتور لابتيف</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>إخطار باستلام شهادة عدم الممانعة المتعلقة بنقل ملكية الأرض إلى شركة أرسنال إيست للتطوير العقاري ( المشتري الجديد النهائي ) ، وإرسال مستندات اتفاقية التطوير، مع طلب التنسيق لاستكمال إجراءات نقل الملكية خلال المدة التعاقدية</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>والمدعية (سي سي ) بهذا الايميل</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>جدول 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>12/05/2026</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>ممثل المدعي عليها 
 والمدعي عليه الثالث 
 فيكتور لابتيف</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع السيد 
 ( خالد أحمد الهاشمي )</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>الرد بشأن الاجتماع مع مبادلة، وإثارة ملاحظات تتعلق باكتمال وتسوية وتسجيل الملكية الحرة للأرض، والتمسك بضرورة استيفاء المستندات والشروط اللازمة لنقل الملكية</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>والمدعية (سي سي ) بهذا الايميل</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>جدول 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>14/05/2026</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع السيد 
 ( خالد أحمد الهاشمي )</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>ممثل المدعي عليها 
 والمدعي عليه الثالث 
 فيكتور لابتيف</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>تأكيد استمرار إجراءات الصفقة وتقديم الاتفاقيات والملاحظات القانونية المعدلة إلى مبادلة، وطلب إصدار شهادة عدم الممانعة النهائية، مع تأكيد قيمة الصفقة النهائية  البالغة 200 مليون درهم وتحديد آلية سدادها بثلاثة شيكات</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>والمدعية (سي سي ) بهذا الايميل</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>جدول 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>19/05/2026</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>ممثل البائع السيد 
 ( خالد أحمد الهاشمي )</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>ممثل المدعي عليها 
 والمدعي عليه الثالث 
 فيكتور لابتيف</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>إرسال إخطار رسمي باستكمال متطلبات الصفقة النهائية والاستعداد لإجراءات نقل الملكية،مرفقًا به شهادة عدم الممانعة واتفاقية التطوير واتفاقية الإنهاء والتنازل، مع طلب استكمال إجراءات التنفيذ والتوقيع</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>والمدعية (سي سي ) بهذا الايميل</t>
         </is>
       </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>جدول 3</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <autoFilter ref="A1:F38"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show the conversation date at the start of every WhatsApp table
Adds a date line above each table, taken from the table title or its
first date row, and expands the title row so its embedded date is visible.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qax4kDvA5VYNQopw9xUKNT
</commit_message>
<xml_diff>
--- a/جداول_الملف.xlsx
+++ b/جداول_الملف.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,12 @@
       <b val="1"/>
       <color rgb="007F7F7F"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -142,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -165,6 +171,9 @@
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -3735,13 +3744,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 1 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 1 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50.5" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -3797,13 +3806,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 2 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 2 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50.5" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -3959,13 +3968,13 @@
       <c r="C19" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 3 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 3 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50.5" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4054,13 +4063,13 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 4 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 4 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50.5" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4147,13 +4156,13 @@
       <c r="C35" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 5 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 5 من الملف  |  التاريخ: 17/02/2026 (تابع للجدول السابق)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="35" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4236,13 +4245,13 @@
       <c r="C44" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 6 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 6 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="50.5" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4373,13 +4382,13 @@
       <c r="C55" s="5" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 7 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 7 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="50.5" customHeight="1">
       <c r="A58" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4546,13 +4555,13 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 8 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 8 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="50.5" customHeight="1">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4677,13 +4686,13 @@
       <c r="C81" s="5" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 9 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 9 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="50.5" customHeight="1">
       <c r="A84" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -4889,13 +4898,13 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 10 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 10 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="50.5" customHeight="1">
       <c r="A101" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5091,13 +5100,13 @@
       <c r="C114" s="5" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 11 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 11 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="50.5" customHeight="1">
       <c r="A117" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5219,13 +5228,13 @@
       <c r="C125" s="5" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 12 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 12 من الملف  |  التاريخ: 17/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="50.5" customHeight="1">
       <c r="A128" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5411,13 +5420,13 @@
       <c r="C141" s="5" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 13 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 13 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="50.5" customHeight="1">
       <c r="A144" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5575,13 +5584,13 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 14 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
+      <c r="A156" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 14 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="50.5" customHeight="1">
       <c r="A157" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5683,13 +5692,13 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 15 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 15 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="50.5" customHeight="1">
       <c r="A166" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5810,13 +5819,13 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 16 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
+      <c r="A175" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 16 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="50.5" customHeight="1">
       <c r="A176" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -5972,13 +5981,13 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 17 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
+      <c r="A188" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 17 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="50.5" customHeight="1">
       <c r="A189" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6083,13 +6092,13 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 18 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
+      <c r="A197" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 18 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="50.5" customHeight="1">
       <c r="A198" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6217,13 +6226,13 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 19 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
+      <c r="A208" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 19 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="50.5" customHeight="1">
       <c r="A209" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6337,13 +6346,13 @@
       <c r="C216" s="5" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 20 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
+      <c r="A218" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 20 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="50.5" customHeight="1">
       <c r="A219" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6443,13 +6452,13 @@
       <c r="C225" s="5" t="n"/>
     </row>
     <row r="227">
-      <c r="A227" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 21 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
+      <c r="A227" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 21 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="50.5" customHeight="1">
       <c r="A228" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6567,13 +6576,13 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 22 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
+      <c r="A238" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 22 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="50.5" customHeight="1">
       <c r="A239" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6716,13 +6725,13 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 23 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
+      <c r="A250" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 23 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="50.5" customHeight="1">
       <c r="A251" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6898,13 +6907,13 @@
       <c r="C263" s="5" t="n"/>
     </row>
     <row r="265">
-      <c r="A265" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 24 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
+      <c r="A265" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 24 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="50.5" customHeight="1">
       <c r="A266" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -6985,13 +6994,13 @@
       <c r="C271" s="5" t="n"/>
     </row>
     <row r="273">
-      <c r="A273" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 25 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
+      <c r="A273" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 25 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="50.5" customHeight="1">
       <c r="A274" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7118,13 +7127,13 @@
       <c r="C282" s="5" t="n"/>
     </row>
     <row r="284">
-      <c r="A284" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 26 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
+      <c r="A284" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 26 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="50.5" customHeight="1">
       <c r="A285" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7242,13 +7251,13 @@
       <c r="C292" s="5" t="n"/>
     </row>
     <row r="294">
-      <c r="A294" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 27 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
+      <c r="A294" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 27 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="50.5" customHeight="1">
       <c r="A295" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7371,13 +7380,13 @@
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 28 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
+      <c r="A304" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 28 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="50.5" customHeight="1">
       <c r="A305" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7511,13 +7520,13 @@
       <c r="C314" s="5" t="n"/>
     </row>
     <row r="316">
-      <c r="A316" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 29 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="317">
+      <c r="A316" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 29 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="50.5" customHeight="1">
       <c r="A317" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7601,13 +7610,13 @@
       <c r="C322" s="5" t="n"/>
     </row>
     <row r="324">
-      <c r="A324" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 30 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
+      <c r="A324" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 30 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="50.5" customHeight="1">
       <c r="A325" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7719,13 +7728,13 @@
       <c r="C332" s="5" t="n"/>
     </row>
     <row r="334">
-      <c r="A334" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 31 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="335">
+      <c r="A334" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 31 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="50.5" customHeight="1">
       <c r="A335" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7814,13 +7823,13 @@
       <c r="C341" s="5" t="n"/>
     </row>
     <row r="343">
-      <c r="A343" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 32 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
+      <c r="A343" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 32 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="50.5" customHeight="1">
       <c r="A344" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -7909,13 +7918,13 @@
       <c r="C349" s="5" t="n"/>
     </row>
     <row r="351">
-      <c r="A351" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 33 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
+      <c r="A351" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 33 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="352" ht="50.5" customHeight="1">
       <c r="A352" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8035,13 +8044,13 @@
       <c r="C360" s="5" t="n"/>
     </row>
     <row r="362">
-      <c r="A362" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 34 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="363">
+      <c r="A362" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 34 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="363" ht="50.5" customHeight="1">
       <c r="A363" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8207,13 +8216,13 @@
       <c r="C374" s="5" t="n"/>
     </row>
     <row r="376">
-      <c r="A376" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 35 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="377">
+      <c r="A376" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 35 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="50.5" customHeight="1">
       <c r="A377" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8339,13 +8348,13 @@
       <c r="C385" s="5" t="n"/>
     </row>
     <row r="387">
-      <c r="A387" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 36 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
+      <c r="A387" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 36 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="388" ht="50.5" customHeight="1">
       <c r="A388" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8439,13 +8448,13 @@
       <c r="C394" s="5" t="n"/>
     </row>
     <row r="396">
-      <c r="A396" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 37 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="397">
+      <c r="A396" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 37 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="397" ht="50.5" customHeight="1">
       <c r="A397" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8556,13 +8565,13 @@
       <c r="C404" s="5" t="n"/>
     </row>
     <row r="406">
-      <c r="A406" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 38 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="407">
+      <c r="A406" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 38 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="407" ht="50.5" customHeight="1">
       <c r="A407" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8674,13 +8683,13 @@
       </c>
     </row>
     <row r="416">
-      <c r="A416" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 39 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="417">
+      <c r="A416" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 39 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="417" ht="50.5" customHeight="1">
       <c r="A417" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8825,13 +8834,13 @@
       </c>
     </row>
     <row r="428">
-      <c r="A428" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 40 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="429">
+      <c r="A428" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 40 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="429" ht="50.5" customHeight="1">
       <c r="A429" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -8971,13 +8980,13 @@
       <c r="C438" s="5" t="n"/>
     </row>
     <row r="440">
-      <c r="A440" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 41 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="441">
+      <c r="A440" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 41 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="441" ht="50.5" customHeight="1">
       <c r="A441" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -9128,13 +9137,13 @@
       <c r="C451" s="5" t="n"/>
     </row>
     <row r="453">
-      <c r="A453" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 42 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="454">
+      <c r="A453" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 42 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="454" ht="50.5" customHeight="1">
       <c r="A454" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -9265,13 +9274,13 @@
       </c>
     </row>
     <row r="464">
-      <c r="A464" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 43 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="465">
+      <c r="A464" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 43 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="465" ht="50.5" customHeight="1">
       <c r="A465" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -9439,13 +9448,13 @@
       </c>
     </row>
     <row r="478">
-      <c r="A478" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 44 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="479">
+      <c r="A478" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 44 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="479" ht="50.5" customHeight="1">
       <c r="A479" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -9576,13 +9585,13 @@
       <c r="C488" s="5" t="n"/>
     </row>
     <row r="490">
-      <c r="A490" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 45 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="491">
+      <c r="A490" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 45 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="491" ht="50.5" customHeight="1">
       <c r="A491" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -9733,13 +9742,13 @@
       <c r="C501" s="5" t="n"/>
     </row>
     <row r="503">
-      <c r="A503" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 46 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="504">
+      <c r="A503" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 46 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="504" ht="50.5" customHeight="1">
       <c r="A504" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -9831,13 +9840,13 @@
       <c r="C509" s="5" t="n"/>
     </row>
     <row r="511">
-      <c r="A511" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 47 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="512">
+      <c r="A511" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 47 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="512" ht="50.5" customHeight="1">
       <c r="A512" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -10005,13 +10014,13 @@
       </c>
     </row>
     <row r="525">
-      <c r="A525" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 48 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="526">
+      <c r="A525" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 48 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="526" ht="50.5" customHeight="1">
       <c r="A526" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -10138,13 +10147,13 @@
       <c r="C534" s="5" t="n"/>
     </row>
     <row r="536">
-      <c r="A536" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 49 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="537">
+      <c r="A536" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 49 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="537" ht="50.5" customHeight="1">
       <c r="A537" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب "آر كي/أرسنال
@@ -10231,13 +10240,13 @@
       </c>
     </row>
     <row r="544">
-      <c r="A544" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 50 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="545">
+      <c r="A544" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 50 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="545" ht="35" customHeight="1">
       <c r="A545" s="8" t="inlineStr">
         <is>
           <t>حادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -10380,13 +10389,13 @@
       </c>
     </row>
     <row r="556">
-      <c r="A556" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 51 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="557">
+      <c r="A556" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 51 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="557" ht="35" customHeight="1">
       <c r="A557" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -10502,13 +10511,13 @@
       </c>
     </row>
     <row r="566">
-      <c r="A566" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 52 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="567">
+      <c r="A566" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 52 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="567" ht="35" customHeight="1">
       <c r="A567" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -10669,13 +10678,13 @@
       </c>
     </row>
     <row r="580">
-      <c r="A580" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 53 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="581">
+      <c r="A580" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 53 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="581" ht="35" customHeight="1">
       <c r="A581" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -10817,13 +10826,13 @@
       <c r="C591" s="5" t="n"/>
     </row>
     <row r="593">
-      <c r="A593" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 54 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="594">
+      <c r="A593" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 54 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="594" ht="35" customHeight="1">
       <c r="A594" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -10904,13 +10913,13 @@
       </c>
     </row>
     <row r="601">
-      <c r="A601" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 55 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="602">
+      <c r="A601" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 55 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="602" ht="35" customHeight="1">
       <c r="A602" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11020,13 +11029,13 @@
       </c>
     </row>
     <row r="611">
-      <c r="A611" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 56 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="612">
+      <c r="A611" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 56 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="612" ht="35" customHeight="1">
       <c r="A612" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11163,13 +11172,13 @@
       </c>
     </row>
     <row r="623">
-      <c r="A623" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 57 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="624">
+      <c r="A623" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 57 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="624" ht="35" customHeight="1">
       <c r="A624" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11316,13 +11325,13 @@
       </c>
     </row>
     <row r="636">
-      <c r="A636" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 58 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="637">
+      <c r="A636" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 58 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="637" ht="35" customHeight="1">
       <c r="A637" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11456,13 +11465,13 @@
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 59 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="649">
+      <c r="A648" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 59 من الملف  |  التاريخ: 18/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="649" ht="35" customHeight="1">
       <c r="A649" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11568,13 +11577,13 @@
       </c>
     </row>
     <row r="658">
-      <c r="A658" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 60 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="659">
+      <c r="A658" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 60 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="659" ht="35" customHeight="1">
       <c r="A659" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11720,13 +11729,13 @@
       <c r="C669" s="5" t="n"/>
     </row>
     <row r="671">
-      <c r="A671" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 61 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="672">
+      <c r="A671" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 61 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="672" ht="35" customHeight="1">
       <c r="A672" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -11860,13 +11869,13 @@
       </c>
     </row>
     <row r="683">
-      <c r="A683" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 62 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="684">
+      <c r="A683" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 62 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="684" ht="35" customHeight="1">
       <c r="A684" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12012,13 +12021,13 @@
       <c r="C694" s="5" t="n"/>
     </row>
     <row r="696">
-      <c r="A696" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 63 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="697">
+      <c r="A696" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 63 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="697" ht="35" customHeight="1">
       <c r="A697" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12155,13 +12164,13 @@
       </c>
     </row>
     <row r="708">
-      <c r="A708" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 64 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="709">
+      <c r="A708" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 64 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="709" ht="35" customHeight="1">
       <c r="A709" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12280,13 +12289,13 @@
       <c r="C717" s="5" t="n"/>
     </row>
     <row r="719">
-      <c r="A719" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 65 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="720">
+      <c r="A719" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 65 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="720" ht="35" customHeight="1">
       <c r="A720" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12432,13 +12441,13 @@
       </c>
     </row>
     <row r="732">
-      <c r="A732" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 66 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="733">
+      <c r="A732" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 66 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="733" ht="35" customHeight="1">
       <c r="A733" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12557,13 +12566,13 @@
       </c>
     </row>
     <row r="743">
-      <c r="A743" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 67 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="744">
+      <c r="A743" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 67 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="744" ht="35" customHeight="1">
       <c r="A744" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12683,13 +12692,13 @@
       <c r="C752" s="5" t="n"/>
     </row>
     <row r="754">
-      <c r="A754" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 68 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="755">
+      <c r="A754" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 68 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="755" ht="35" customHeight="1">
       <c r="A755" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12779,13 +12788,13 @@
       <c r="C761" s="5" t="n"/>
     </row>
     <row r="763">
-      <c r="A763" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 69 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="764">
+      <c r="A763" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 69 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="764" ht="35" customHeight="1">
       <c r="A764" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -12907,13 +12916,13 @@
       </c>
     </row>
     <row r="774">
-      <c r="A774" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 70 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="775">
+      <c r="A774" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 70 من الملف  |  التاريخ: 19/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="775" ht="35" customHeight="1">
       <c r="A775" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -13053,13 +13062,13 @@
       <c r="C785" s="5" t="n"/>
     </row>
     <row r="787">
-      <c r="A787" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 71 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="788">
+      <c r="A787" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 71 من الملف  |  التاريخ: 23/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="788" ht="35" customHeight="1">
       <c r="A788" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -13178,13 +13187,13 @@
       <c r="E795" s="4" t="n"/>
     </row>
     <row r="797">
-      <c r="A797" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 72 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="798">
+      <c r="A797" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 72 من الملف  |  التاريخ: 23/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="798" ht="35" customHeight="1">
       <c r="A798" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -13338,13 +13347,13 @@
       <c r="E807" s="4" t="n"/>
     </row>
     <row r="809">
-      <c r="A809" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 73 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="810">
+      <c r="A809" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 73 من الملف  |  التاريخ: 23/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="810" ht="35" customHeight="1">
       <c r="A810" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -13452,13 +13461,13 @@
       </c>
     </row>
     <row r="819">
-      <c r="A819" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 74 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="820">
+      <c r="A819" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 74 من الملف  |  التاريخ: 24/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="820" ht="35" customHeight="1">
       <c r="A820" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -13628,13 +13637,13 @@
       </c>
     </row>
     <row r="834">
-      <c r="A834" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 75 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="835">
+      <c r="A834" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 75 من الملف  |  التاريخ: 24/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="835" ht="35" customHeight="1">
       <c r="A835" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -13734,13 +13743,13 @@
       </c>
     </row>
     <row r="843">
-      <c r="A843" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 76 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="844">
+      <c r="A843" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 76 من الملف  |  التاريخ: 24/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="844" ht="35" customHeight="1">
       <c r="A844" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -13900,13 +13909,13 @@
       </c>
     </row>
     <row r="857">
-      <c r="A857" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 77 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="858">
+      <c r="A857" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 77 من الملف  |  التاريخ: 24/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="858" ht="35" customHeight="1">
       <c r="A858" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14094,13 +14103,13 @@
       </c>
     </row>
     <row r="873">
-      <c r="A873" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 78 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="874">
+      <c r="A873" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 78 من الملف  |  التاريخ: 24/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="874" ht="35" customHeight="1">
       <c r="A874" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14275,13 +14284,13 @@
       </c>
     </row>
     <row r="888">
-      <c r="A888" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 79 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="889">
+      <c r="A888" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 79 من الملف  |  التاريخ: 24/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="889" ht="35" customHeight="1">
       <c r="A889" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14409,13 +14418,13 @@
       </c>
     </row>
     <row r="900">
-      <c r="A900" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 80 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="901">
+      <c r="A900" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 80 من الملف  |  التاريخ: 26/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="901" ht="35" customHeight="1">
       <c r="A901" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14574,13 +14583,13 @@
       </c>
     </row>
     <row r="914">
-      <c r="A914" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 81 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="915">
+      <c r="A914" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 81 من الملف  |  التاريخ: 27/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="915" ht="35" customHeight="1">
       <c r="A915" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14719,13 +14728,13 @@
       </c>
     </row>
     <row r="926">
-      <c r="A926" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 82 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="927">
+      <c r="A926" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 82 من الملف  |  التاريخ: 27/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="927" ht="35" customHeight="1">
       <c r="A927" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14873,13 +14882,13 @@
       </c>
     </row>
     <row r="939">
-      <c r="A939" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 83 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="940">
+      <c r="A939" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 83 من الملف  |  التاريخ: 01/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="940" ht="35" customHeight="1">
       <c r="A940" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -14956,13 +14965,13 @@
       </c>
     </row>
     <row r="947">
-      <c r="A947" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 84 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="948">
+      <c r="A947" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 84 من الملف  |  التاريخ: 02/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="948" ht="35" customHeight="1">
       <c r="A948" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15149,13 +15158,13 @@
       </c>
     </row>
     <row r="963">
-      <c r="A963" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 85 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="964">
+      <c r="A963" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 85 من الملف  |  التاريخ: 03/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="964" ht="35" customHeight="1">
       <c r="A964" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15286,13 +15295,13 @@
       <c r="C973" s="5" t="n"/>
     </row>
     <row r="975">
-      <c r="A975" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 86 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="976">
+      <c r="A975" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 86 من الملف  |  التاريخ: 03/03/2026 (تابع للجدول السابق)</t>
+        </is>
+      </c>
+    </row>
+    <row r="976" ht="35" customHeight="1">
       <c r="A976" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15417,13 +15426,13 @@
       </c>
     </row>
     <row r="986">
-      <c r="A986" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 87 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="987">
+      <c r="A986" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 87 من الملف  |  التاريخ: 03/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="987" ht="35" customHeight="1">
       <c r="A987" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15553,13 +15562,13 @@
       <c r="C996" s="5" t="n"/>
     </row>
     <row r="998">
-      <c r="A998" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 88 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="999">
+      <c r="A998" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 88 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="999" ht="35" customHeight="1">
       <c r="A999" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15668,13 +15677,13 @@
       </c>
     </row>
     <row r="1008">
-      <c r="A1008" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 89 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1009">
+      <c r="A1008" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 89 من الملف  |  التاريخ: 04/03/2026 (تابع للجدول السابق)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009" ht="35" customHeight="1">
       <c r="A1009" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15790,13 +15799,13 @@
       </c>
     </row>
     <row r="1018">
-      <c r="A1018" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 90 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1019">
+      <c r="A1018" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 90 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019" ht="35" customHeight="1">
       <c r="A1019" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -15928,13 +15937,13 @@
       </c>
     </row>
     <row r="1030">
-      <c r="A1030" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 91 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1031">
+      <c r="A1030" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 91 من الملف  |  التاريخ: 04/03/2026 (تابع للجدول السابق)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031" ht="35" customHeight="1">
       <c r="A1031" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -16090,13 +16099,13 @@
       </c>
     </row>
     <row r="1043">
-      <c r="A1043" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 92 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1044">
+      <c r="A1043" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 92 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044" ht="35" customHeight="1">
       <c r="A1044" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -16245,13 +16254,13 @@
       </c>
     </row>
     <row r="1056">
-      <c r="A1056" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 93 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1057">
+      <c r="A1056" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 93 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057" ht="35" customHeight="1">
       <c r="A1057" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -16374,13 +16383,13 @@
       </c>
     </row>
     <row r="1067">
-      <c r="A1067" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 94 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1068">
+      <c r="A1067" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 94 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068" ht="35" customHeight="1">
       <c r="A1068" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -16530,13 +16539,13 @@
       </c>
     </row>
     <row r="1080">
-      <c r="A1080" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 95 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1081">
+      <c r="A1080" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 95 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081" ht="35" customHeight="1">
       <c r="A1081" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -16804,13 +16813,13 @@
       </c>
     </row>
     <row r="1102">
-      <c r="A1102" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 96 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1103">
+      <c r="A1102" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 96 من الملف  |  التاريخ: 04/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103" ht="35" customHeight="1">
       <c r="A1103" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -16940,13 +16949,13 @@
       </c>
     </row>
     <row r="1114">
-      <c r="A1114" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 97 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1115">
+      <c r="A1114" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 97 من الملف  |  التاريخ: 05/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115" ht="35" customHeight="1">
       <c r="A1115" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -17088,13 +17097,13 @@
       </c>
     </row>
     <row r="1127">
-      <c r="A1127" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 98 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1128">
+      <c r="A1127" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 98 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128" ht="35" customHeight="1">
       <c r="A1128" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -17213,13 +17222,13 @@
       </c>
     </row>
     <row r="1138">
-      <c r="A1138" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 99 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1139">
+      <c r="A1138" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 99 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139" ht="35" customHeight="1">
       <c r="A1139" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -17355,13 +17364,13 @@
       </c>
     </row>
     <row r="1150">
-      <c r="A1150" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 100 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1151">
+      <c r="A1150" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 100 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151" ht="35" customHeight="1">
       <c r="A1151" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -17501,13 +17510,13 @@
       </c>
     </row>
     <row r="1162">
-      <c r="A1162" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 101 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1163">
+      <c r="A1162" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 101 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163" ht="35" customHeight="1">
       <c r="A1163" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -17682,13 +17691,13 @@
       </c>
     </row>
     <row r="1177">
-      <c r="A1177" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 102 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1178">
+      <c r="A1177" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 102 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178" ht="35" customHeight="1">
       <c r="A1178" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -17860,13 +17869,13 @@
       </c>
     </row>
     <row r="1192">
-      <c r="A1192" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 103 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1193">
+      <c r="A1192" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 103 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193" ht="35" customHeight="1">
       <c r="A1193" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18026,13 +18035,13 @@
       </c>
     </row>
     <row r="1206">
-      <c r="A1206" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 104 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1207">
+      <c r="A1206" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 104 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207" ht="35" customHeight="1">
       <c r="A1207" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18154,13 +18163,13 @@
       </c>
     </row>
     <row r="1217">
-      <c r="A1217" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 105 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1218">
+      <c r="A1217" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 105 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218" ht="35" customHeight="1">
       <c r="A1218" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18291,13 +18300,13 @@
       </c>
     </row>
     <row r="1229">
-      <c r="A1229" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 106 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1230">
+      <c r="A1229" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 106 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230" ht="35" customHeight="1">
       <c r="A1230" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18456,13 +18465,13 @@
       </c>
     </row>
     <row r="1243">
-      <c r="A1243" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 107 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1244">
+      <c r="A1243" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 107 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244" ht="35" customHeight="1">
       <c r="A1244" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18594,13 +18603,13 @@
       </c>
     </row>
     <row r="1255">
-      <c r="A1255" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 108 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1256">
+      <c r="A1255" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 108 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256" ht="35" customHeight="1">
       <c r="A1256" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18785,13 +18794,13 @@
       </c>
     </row>
     <row r="1271">
-      <c r="A1271" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 109 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1272">
+      <c r="A1271" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 109 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272" ht="35" customHeight="1">
       <c r="A1272" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -18940,13 +18949,13 @@
       </c>
     </row>
     <row r="1284">
-      <c r="A1284" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 110 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1285">
+      <c r="A1284" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 110 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285" ht="35" customHeight="1">
       <c r="A1285" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -19084,13 +19093,13 @@
       </c>
     </row>
     <row r="1296">
-      <c r="A1296" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 111 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1297">
+      <c r="A1296" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 111 من الملف  |  التاريخ: 06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297" ht="35" customHeight="1">
       <c r="A1297" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -19266,13 +19275,13 @@
       </c>
     </row>
     <row r="1311">
-      <c r="A1311" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 112 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1312">
+      <c r="A1311" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 112 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312" ht="35" customHeight="1">
       <c r="A1312" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -19416,13 +19425,13 @@
       </c>
     </row>
     <row r="1324">
-      <c r="A1324" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 113 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1325">
+      <c r="A1324" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 113 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325" ht="35" customHeight="1">
       <c r="A1325" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -19575,13 +19584,13 @@
       </c>
     </row>
     <row r="1337">
-      <c r="A1337" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 114 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1338">
+      <c r="A1337" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 114 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338" ht="35" customHeight="1">
       <c r="A1338" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -19695,13 +19704,13 @@
       </c>
     </row>
     <row r="1347">
-      <c r="A1347" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 115 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1348">
+      <c r="A1347" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 115 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348" ht="35" customHeight="1">
       <c r="A1348" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -19885,13 +19894,13 @@
       <c r="E1359" s="4" t="n"/>
     </row>
     <row r="1361">
-      <c r="A1361" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 116 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1362">
+      <c r="A1361" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 116 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362" ht="35" customHeight="1">
       <c r="A1362" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -20065,13 +20074,13 @@
       <c r="E1372" s="4" t="n"/>
     </row>
     <row r="1374">
-      <c r="A1374" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 117 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1375">
+      <c r="A1374" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 117 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375" ht="35" customHeight="1">
       <c r="A1375" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -20267,13 +20276,13 @@
       <c r="E1387" s="4" t="n"/>
     </row>
     <row r="1389">
-      <c r="A1389" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 118 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1390">
+      <c r="A1389" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 118 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390" ht="35" customHeight="1">
       <c r="A1390" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -20356,13 +20365,13 @@
       <c r="E1394" s="4" t="n"/>
     </row>
     <row r="1396">
-      <c r="A1396" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 119 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1397">
+      <c r="A1396" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 119 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397" ht="35" customHeight="1">
       <c r="A1397" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -20485,13 +20494,13 @@
       <c r="E1404" s="4" t="n"/>
     </row>
     <row r="1406">
-      <c r="A1406" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 120 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1407">
+      <c r="A1406" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 120 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407" ht="35" customHeight="1">
       <c r="A1407" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -20628,13 +20637,13 @@
       <c r="E1415" s="4" t="n"/>
     </row>
     <row r="1417">
-      <c r="A1417" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 121 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1418">
+      <c r="A1417" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 121 من الملف  |  التاريخ: 11/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418" ht="35" customHeight="1">
       <c r="A1418" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب  مع آر كيه/ أرسنال
@@ -20782,13 +20791,13 @@
       <c r="E1427" s="4" t="n"/>
     </row>
     <row r="1429">
-      <c r="A1429" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 122 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1430">
+      <c r="A1429" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 122 من الملف  |  التاريخ: 14/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430" ht="35" customHeight="1">
       <c r="A1430" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -20956,13 +20965,13 @@
       </c>
     </row>
     <row r="1444">
-      <c r="A1444" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 123 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1445">
+      <c r="A1444" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 123 من الملف  |  التاريخ: 15/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445" ht="35" customHeight="1">
       <c r="A1445" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -21135,13 +21144,13 @@
       <c r="C1458" s="5" t="n"/>
     </row>
     <row r="1460">
-      <c r="A1460" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 124 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1461">
+      <c r="A1460" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 124 من الملف  |  التاريخ: 18/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461" ht="35" customHeight="1">
       <c r="A1461" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -21272,13 +21281,13 @@
       <c r="C1471" s="4" t="n"/>
     </row>
     <row r="1473">
-      <c r="A1473" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 125 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1474">
+      <c r="A1473" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 125 من الملف  |  التاريخ: 25/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474" ht="35" customHeight="1">
       <c r="A1474" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -21401,13 +21410,13 @@
       </c>
     </row>
     <row r="1484">
-      <c r="A1484" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 126 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1485">
+      <c r="A1484" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 126 من الملف  |  التاريخ: 25/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485" ht="35" customHeight="1">
       <c r="A1485" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -21559,13 +21568,13 @@
       </c>
     </row>
     <row r="1498">
-      <c r="A1498" s="7" t="inlineStr">
-        <is>
-          <t>الجدول رقم 127 من الملف</t>
-        </is>
-      </c>
-    </row>
-    <row r="1499">
+      <c r="A1498" s="10" t="inlineStr">
+        <is>
+          <t>الجدول رقم 127 من الملف  |  التاريخ: 08/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499" ht="35" customHeight="1">
       <c r="A1499" s="8" t="inlineStr">
         <is>
           <t>محادثة عبر تطبيق الواتساب مع آر كيه/ أرسنال
@@ -21703,7 +21712,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="355">
+  <mergeCells count="482">
     <mergeCell ref="A128:C128"/>
     <mergeCell ref="B1355:C1355"/>
     <mergeCell ref="A1445:C1445"/>
@@ -21711,9 +21720,15 @@
     <mergeCell ref="D1371:E1371"/>
     <mergeCell ref="A720:C720"/>
     <mergeCell ref="A891:C891"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A1018:C1018"/>
+    <mergeCell ref="A1162:C1162"/>
+    <mergeCell ref="A428:C428"/>
+    <mergeCell ref="A57:C57"/>
     <mergeCell ref="B802:C802"/>
     <mergeCell ref="D802:E802"/>
     <mergeCell ref="A1447:C1447"/>
+    <mergeCell ref="A857:C857"/>
     <mergeCell ref="A1390:E1390"/>
     <mergeCell ref="B1394:C1394"/>
     <mergeCell ref="A479:C479"/>
@@ -21721,7 +21736,9 @@
     <mergeCell ref="B1387:C1387"/>
     <mergeCell ref="D1387:E1387"/>
     <mergeCell ref="B805:C805"/>
+    <mergeCell ref="A873:C873"/>
     <mergeCell ref="A352:C352"/>
+    <mergeCell ref="A83:C83"/>
     <mergeCell ref="A860:C860"/>
     <mergeCell ref="B1400:C1400"/>
     <mergeCell ref="D1351:E1351"/>
@@ -21729,15 +21746,23 @@
     <mergeCell ref="A639:C639"/>
     <mergeCell ref="A614:C614"/>
     <mergeCell ref="A789:B789"/>
+    <mergeCell ref="A334:C334"/>
     <mergeCell ref="C789:D789"/>
     <mergeCell ref="D1393:E1393"/>
     <mergeCell ref="A948:C948"/>
     <mergeCell ref="A837:C837"/>
     <mergeCell ref="A929:C929"/>
+    <mergeCell ref="A914:C914"/>
+    <mergeCell ref="A708:C708"/>
+    <mergeCell ref="A238:C238"/>
     <mergeCell ref="A1471:C1471"/>
+    <mergeCell ref="A1008:C1008"/>
     <mergeCell ref="B1411:C1411"/>
     <mergeCell ref="A1230:C1230"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A1153:C1153"/>
+    <mergeCell ref="A265:C265"/>
+    <mergeCell ref="A1324:C1324"/>
     <mergeCell ref="D1421:E1421"/>
     <mergeCell ref="A1376:B1376"/>
     <mergeCell ref="C1376:D1376"/>
@@ -21746,20 +21771,27 @@
     <mergeCell ref="A1019:C1019"/>
     <mergeCell ref="C1363:D1363"/>
     <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A1255:C1255"/>
     <mergeCell ref="A1021:C1021"/>
     <mergeCell ref="A266:C266"/>
+    <mergeCell ref="A1192:C1192"/>
     <mergeCell ref="A1463:C1463"/>
     <mergeCell ref="D805:E805"/>
     <mergeCell ref="A1375:E1375"/>
+    <mergeCell ref="A1406:E1406"/>
+    <mergeCell ref="A197:C197"/>
     <mergeCell ref="B1424:C1424"/>
     <mergeCell ref="D1424:E1424"/>
     <mergeCell ref="D807:E807"/>
+    <mergeCell ref="A658:C658"/>
     <mergeCell ref="A84:C84"/>
     <mergeCell ref="B1401:C1401"/>
     <mergeCell ref="A1399:E1399"/>
     <mergeCell ref="D1401:E1401"/>
     <mergeCell ref="A876:C876"/>
+    <mergeCell ref="A1374:E1374"/>
     <mergeCell ref="D1367:E1367"/>
+    <mergeCell ref="A188:C188"/>
     <mergeCell ref="A940:C940"/>
     <mergeCell ref="A989:C989"/>
     <mergeCell ref="A976:C976"/>
@@ -21769,23 +21801,29 @@
     <mergeCell ref="A709:C709"/>
     <mergeCell ref="A684:C684"/>
     <mergeCell ref="A1461:C1461"/>
+    <mergeCell ref="A1138:C1138"/>
     <mergeCell ref="A1485:C1485"/>
     <mergeCell ref="A711:C711"/>
     <mergeCell ref="A686:C686"/>
     <mergeCell ref="B1427:C1427"/>
+    <mergeCell ref="A490:C490"/>
     <mergeCell ref="D793:E793"/>
     <mergeCell ref="B791:C791"/>
     <mergeCell ref="B1356:C1356"/>
     <mergeCell ref="D1385:E1385"/>
     <mergeCell ref="D801:E801"/>
     <mergeCell ref="D795:E795"/>
+    <mergeCell ref="A1389:E1389"/>
     <mergeCell ref="D1422:E1422"/>
     <mergeCell ref="B1358:C1358"/>
     <mergeCell ref="A1327:C1327"/>
+    <mergeCell ref="A1498:C1498"/>
+    <mergeCell ref="A566:C566"/>
     <mergeCell ref="B1351:C1351"/>
     <mergeCell ref="A397:C397"/>
     <mergeCell ref="A1093:C1093"/>
     <mergeCell ref="A1220:C1220"/>
+    <mergeCell ref="A503:C503"/>
     <mergeCell ref="B1382:C1382"/>
     <mergeCell ref="A1108:C1108"/>
     <mergeCell ref="D1411:E1411"/>
@@ -21797,22 +21835,36 @@
     <mergeCell ref="D1412:E1412"/>
     <mergeCell ref="A661:C661"/>
     <mergeCell ref="A755:C755"/>
+    <mergeCell ref="A819:C819"/>
     <mergeCell ref="A757:C757"/>
+    <mergeCell ref="A1177:C1177"/>
+    <mergeCell ref="A1484:C1484"/>
+    <mergeCell ref="A343:C343"/>
     <mergeCell ref="A1340:C1340"/>
     <mergeCell ref="A1398:B1398"/>
     <mergeCell ref="B1366:C1366"/>
     <mergeCell ref="C1398:D1398"/>
     <mergeCell ref="B1353:C1353"/>
+    <mergeCell ref="A218:C218"/>
+    <mergeCell ref="A1271:C1271"/>
+    <mergeCell ref="A316:C316"/>
     <mergeCell ref="A1081:C1081"/>
     <mergeCell ref="B1368:C1368"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A797:E797"/>
     <mergeCell ref="D803:E803"/>
     <mergeCell ref="B1370:C1370"/>
+    <mergeCell ref="A376:C376"/>
     <mergeCell ref="A1083:C1083"/>
     <mergeCell ref="D1386:E1386"/>
     <mergeCell ref="B1422:C1422"/>
+    <mergeCell ref="A71:C71"/>
     <mergeCell ref="B1372:C1372"/>
     <mergeCell ref="D1415:E1415"/>
+    <mergeCell ref="A1206:C1206"/>
+    <mergeCell ref="A926:C926"/>
     <mergeCell ref="A1391:B1391"/>
+    <mergeCell ref="A165:C165"/>
     <mergeCell ref="C1391:D1391"/>
     <mergeCell ref="A407:C407"/>
     <mergeCell ref="A874:C874"/>
@@ -21821,22 +21873,34 @@
     <mergeCell ref="A1457:C1457"/>
     <mergeCell ref="A569:C569"/>
     <mergeCell ref="A1493:C1493"/>
+    <mergeCell ref="A732:C732"/>
     <mergeCell ref="A903:C903"/>
+    <mergeCell ref="A1030:C1030"/>
     <mergeCell ref="A1272:C1272"/>
     <mergeCell ref="A967:C967"/>
     <mergeCell ref="A1501:C1501"/>
     <mergeCell ref="A733:C733"/>
     <mergeCell ref="A1419:B1419"/>
     <mergeCell ref="B1385:C1385"/>
+    <mergeCell ref="A351:C351"/>
+    <mergeCell ref="A1056:C1056"/>
+    <mergeCell ref="A1127:C1127"/>
     <mergeCell ref="A239:C239"/>
+    <mergeCell ref="A1043:C1043"/>
     <mergeCell ref="A1285:C1285"/>
+    <mergeCell ref="A464:C464"/>
     <mergeCell ref="A651:C651"/>
     <mergeCell ref="A822:C822"/>
     <mergeCell ref="A1408:B1408"/>
+    <mergeCell ref="A1229:C1229"/>
+    <mergeCell ref="A601:C601"/>
     <mergeCell ref="A219:C219"/>
     <mergeCell ref="B1369:C1369"/>
     <mergeCell ref="B1413:C1413"/>
     <mergeCell ref="A1232:C1232"/>
+    <mergeCell ref="A900:C900"/>
+    <mergeCell ref="A250:C250"/>
+    <mergeCell ref="A998:C998"/>
     <mergeCell ref="A777:C777"/>
     <mergeCell ref="A942:C942"/>
     <mergeCell ref="A1209:C1209"/>
@@ -21844,6 +21908,8 @@
     <mergeCell ref="A537:C537"/>
     <mergeCell ref="A189:C189"/>
     <mergeCell ref="A512:C512"/>
+    <mergeCell ref="A683:C683"/>
+    <mergeCell ref="A754:C754"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="B1357:C1357"/>
     <mergeCell ref="D1357:E1357"/>
@@ -21858,37 +21924,56 @@
     <mergeCell ref="A1193:C1193"/>
     <mergeCell ref="A894:C894"/>
     <mergeCell ref="A1003:C1003"/>
+    <mergeCell ref="A888:C888"/>
+    <mergeCell ref="A304:C304"/>
+    <mergeCell ref="A1130:C1130"/>
     <mergeCell ref="A1059:C1059"/>
-    <mergeCell ref="A1130:C1130"/>
+    <mergeCell ref="A986:C986"/>
+    <mergeCell ref="A396:C396"/>
     <mergeCell ref="A936:C936"/>
     <mergeCell ref="B806:C806"/>
+    <mergeCell ref="A1067:C1067"/>
     <mergeCell ref="D1370:E1370"/>
     <mergeCell ref="A917:C917"/>
     <mergeCell ref="A1430:C1430"/>
+    <mergeCell ref="A227:C227"/>
     <mergeCell ref="D1372:E1372"/>
     <mergeCell ref="A335:C335"/>
     <mergeCell ref="B801:C801"/>
+    <mergeCell ref="A556:C556"/>
     <mergeCell ref="A1350:E1350"/>
     <mergeCell ref="A950:C950"/>
     <mergeCell ref="A251:C251"/>
+    <mergeCell ref="A116:C116"/>
     <mergeCell ref="A545:C545"/>
+    <mergeCell ref="A843:C843"/>
+    <mergeCell ref="A324:C324"/>
     <mergeCell ref="A1299:C1299"/>
+    <mergeCell ref="A416:C416"/>
     <mergeCell ref="A780:C780"/>
+    <mergeCell ref="A774:C774"/>
     <mergeCell ref="A117:C117"/>
     <mergeCell ref="A1314:C1314"/>
     <mergeCell ref="A788:E788"/>
     <mergeCell ref="D1365:E1365"/>
     <mergeCell ref="A1105:C1105"/>
+    <mergeCell ref="A1080:C1080"/>
     <mergeCell ref="D1423:E1423"/>
     <mergeCell ref="B804:C804"/>
     <mergeCell ref="B1421:C1421"/>
     <mergeCell ref="A429:C429"/>
+    <mergeCell ref="A1243:C1243"/>
+    <mergeCell ref="A963:C963"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A208:C208"/>
     <mergeCell ref="A1009:C1009"/>
     <mergeCell ref="B793:C793"/>
     <mergeCell ref="A1465:C1465"/>
+    <mergeCell ref="A406:C406"/>
     <mergeCell ref="A775:C775"/>
     <mergeCell ref="A1244:C1244"/>
     <mergeCell ref="B1412:C1412"/>
+    <mergeCell ref="A1296:C1296"/>
     <mergeCell ref="B1378:C1378"/>
     <mergeCell ref="D1378:E1378"/>
     <mergeCell ref="D1380:E1380"/>
@@ -21909,18 +21994,24 @@
     <mergeCell ref="B1371:C1371"/>
     <mergeCell ref="A198:C198"/>
     <mergeCell ref="A654:C654"/>
+    <mergeCell ref="A719:C719"/>
     <mergeCell ref="A1377:E1377"/>
     <mergeCell ref="B794:C794"/>
     <mergeCell ref="D794:E794"/>
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="A209:C209"/>
     <mergeCell ref="A274:C274"/>
+    <mergeCell ref="A743:C743"/>
     <mergeCell ref="A1246:C1246"/>
     <mergeCell ref="A672:C672"/>
+    <mergeCell ref="A536:C536"/>
+    <mergeCell ref="A511:C511"/>
+    <mergeCell ref="A809:C809"/>
     <mergeCell ref="A1070:C1070"/>
     <mergeCell ref="B1415:C1415"/>
     <mergeCell ref="A1312:C1312"/>
     <mergeCell ref="A649:C649"/>
+    <mergeCell ref="A947:C947"/>
     <mergeCell ref="A798:E798"/>
     <mergeCell ref="A567:C567"/>
     <mergeCell ref="D1381:E1381"/>
@@ -21929,8 +22020,10 @@
     <mergeCell ref="A800:E800"/>
     <mergeCell ref="B1410:C1410"/>
     <mergeCell ref="D1410:E1410"/>
+    <mergeCell ref="A787:E787"/>
     <mergeCell ref="A1165:C1165"/>
     <mergeCell ref="D1382:E1382"/>
+    <mergeCell ref="A440:C440"/>
     <mergeCell ref="D1425:E1425"/>
     <mergeCell ref="A896:C896"/>
     <mergeCell ref="A377:C377"/>
@@ -21938,9 +22031,12 @@
     <mergeCell ref="A504:C504"/>
     <mergeCell ref="A491:C491"/>
     <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A362:C362"/>
     <mergeCell ref="A1403:E1403"/>
     <mergeCell ref="A1397:E1397"/>
     <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A1347:E1347"/>
+    <mergeCell ref="A580:C580"/>
     <mergeCell ref="B1365:C1365"/>
     <mergeCell ref="D1394:E1394"/>
     <mergeCell ref="A987:C987"/>
@@ -21948,22 +22044,28 @@
     <mergeCell ref="A674:C674"/>
     <mergeCell ref="A388:C388"/>
     <mergeCell ref="A581:C581"/>
+    <mergeCell ref="A1311:C1311"/>
     <mergeCell ref="A1115:C1115"/>
+    <mergeCell ref="A611:C611"/>
+    <mergeCell ref="A1102:C1102"/>
     <mergeCell ref="A285:C285"/>
-    <mergeCell ref="D1400:E1400"/>
     <mergeCell ref="A1338:C1338"/>
     <mergeCell ref="A583:C583"/>
+    <mergeCell ref="D1400:E1400"/>
     <mergeCell ref="A1117:C1117"/>
     <mergeCell ref="A1392:E1392"/>
+    <mergeCell ref="A975:C975"/>
     <mergeCell ref="B795:C795"/>
     <mergeCell ref="A295:C295"/>
     <mergeCell ref="A764:C764"/>
     <mergeCell ref="D792:E792"/>
+    <mergeCell ref="A143:C143"/>
     <mergeCell ref="A1031:C1031"/>
     <mergeCell ref="A441:C441"/>
     <mergeCell ref="A810:C810"/>
     <mergeCell ref="A790:E790"/>
     <mergeCell ref="A1046:C1046"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A812:C812"/>
     <mergeCell ref="A799:B799"/>
     <mergeCell ref="A1418:E1418"/>
@@ -21971,6 +22073,7 @@
     <mergeCell ref="A1091:C1091"/>
     <mergeCell ref="A363:C363"/>
     <mergeCell ref="B1386:C1386"/>
+    <mergeCell ref="A273:C273"/>
     <mergeCell ref="D1402:E1402"/>
     <mergeCell ref="B1352:C1352"/>
     <mergeCell ref="D1352:E1352"/>
@@ -21979,29 +22082,40 @@
     <mergeCell ref="B1381:C1381"/>
     <mergeCell ref="A1123:C1123"/>
     <mergeCell ref="A1044:C1044"/>
+    <mergeCell ref="A156:C156"/>
     <mergeCell ref="B1383:C1383"/>
     <mergeCell ref="A454:C454"/>
     <mergeCell ref="D1383:E1383"/>
+    <mergeCell ref="A525:C525"/>
+    <mergeCell ref="A696:C696"/>
     <mergeCell ref="A889:C889"/>
+    <mergeCell ref="A1473:C1473"/>
     <mergeCell ref="A612:C612"/>
     <mergeCell ref="A858:C858"/>
+    <mergeCell ref="A1217:C1217"/>
     <mergeCell ref="A820:C820"/>
     <mergeCell ref="A157:C157"/>
+    <mergeCell ref="A284:C284"/>
     <mergeCell ref="C799:D799"/>
     <mergeCell ref="A958:C958"/>
     <mergeCell ref="A1256:C1256"/>
     <mergeCell ref="A1057:C1057"/>
     <mergeCell ref="A1258:C1258"/>
     <mergeCell ref="D806:E806"/>
+    <mergeCell ref="A1429:C1429"/>
     <mergeCell ref="A1499:C1499"/>
     <mergeCell ref="A317:C317"/>
     <mergeCell ref="A602:C602"/>
     <mergeCell ref="A1409:E1409"/>
     <mergeCell ref="A596:C596"/>
     <mergeCell ref="C1349:D1349"/>
+    <mergeCell ref="A1396:E1396"/>
+    <mergeCell ref="A175:C175"/>
     <mergeCell ref="A604:C604"/>
     <mergeCell ref="A744:C744"/>
+    <mergeCell ref="A1361:E1361"/>
     <mergeCell ref="D1358:E1358"/>
+    <mergeCell ref="A671:C671"/>
     <mergeCell ref="A1348:E1348"/>
     <mergeCell ref="A1420:E1420"/>
     <mergeCell ref="A735:C735"/>
@@ -22014,41 +22128,63 @@
     <mergeCell ref="A526:C526"/>
     <mergeCell ref="A697:C697"/>
     <mergeCell ref="A1474:C1474"/>
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="A305:C305"/>
     <mergeCell ref="A1218:C1218"/>
     <mergeCell ref="A1489:C1489"/>
+    <mergeCell ref="A1460:C1460"/>
     <mergeCell ref="A699:C699"/>
     <mergeCell ref="A626:C626"/>
     <mergeCell ref="A101:C101"/>
+    <mergeCell ref="A294:C294"/>
     <mergeCell ref="A465:C465"/>
+    <mergeCell ref="A636:C636"/>
+    <mergeCell ref="A763:C763"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A999:C999"/>
     <mergeCell ref="A1195:C1195"/>
     <mergeCell ref="A1297:C1297"/>
+    <mergeCell ref="A1284:C1284"/>
     <mergeCell ref="D1366:E1366"/>
     <mergeCell ref="B1402:C1402"/>
     <mergeCell ref="D1353:E1353"/>
+    <mergeCell ref="A1417:E1417"/>
     <mergeCell ref="D1368:E1368"/>
     <mergeCell ref="B1404:C1404"/>
+    <mergeCell ref="A127:C127"/>
     <mergeCell ref="B1379:C1379"/>
     <mergeCell ref="D1379:E1379"/>
     <mergeCell ref="A176:C176"/>
+    <mergeCell ref="A1444:C1444"/>
+    <mergeCell ref="A648:C648"/>
+    <mergeCell ref="A387:C387"/>
     <mergeCell ref="A1139:C1139"/>
+    <mergeCell ref="A939:C939"/>
+    <mergeCell ref="A623:C623"/>
+    <mergeCell ref="A1362:E1362"/>
     <mergeCell ref="A1437:C1437"/>
-    <mergeCell ref="A1362:E1362"/>
+    <mergeCell ref="A1114:C1114"/>
+    <mergeCell ref="A1150:C1150"/>
+    <mergeCell ref="A1337:C1337"/>
     <mergeCell ref="A1141:C1141"/>
     <mergeCell ref="A1364:E1364"/>
+    <mergeCell ref="A478:C478"/>
+    <mergeCell ref="A453:C453"/>
     <mergeCell ref="A624:C624"/>
     <mergeCell ref="B792:C792"/>
     <mergeCell ref="D1356:E1356"/>
     <mergeCell ref="B807:C807"/>
     <mergeCell ref="A1068:C1068"/>
     <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A834:C834"/>
+    <mergeCell ref="A100:C100"/>
     <mergeCell ref="A594:C594"/>
     <mergeCell ref="A1363:B1363"/>
+    <mergeCell ref="A544:C544"/>
+    <mergeCell ref="A344:C344"/>
     <mergeCell ref="A1432:C1432"/>
-    <mergeCell ref="A344:C344"/>
     <mergeCell ref="C1419:D1419"/>
+    <mergeCell ref="A593:C593"/>
     <mergeCell ref="B1423:C1423"/>
     <mergeCell ref="A927:C927"/>
     <mergeCell ref="A166:C166"/>

</xml_diff>